<commit_message>
chore(import): replace items excel template with provided file
</commit_message>
<xml_diff>
--- a/public/templates/items-import-template.xlsx
+++ b/public/templates/items-import-template.xlsx
@@ -1,41 +1,56 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="22130"/>
   <workbookPr codeName="ThisWorkbook"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dvinskikh.sergey\Desktop\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B99480AC-1259-44F3-8E82-3E912F754EDE}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
     <sheet name="Items" sheetId="1" r:id="rId1"/>
   </sheets>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
-<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
-  <metadataTypes count="1">
-    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
-  </metadataTypes>
-  <futureMetadata name="XLDAPR" count="1">
-    <bk>
-      <extLst>
-        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
-          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
-        </ext>
-      </extLst>
-    </bk>
-  </futureMetadata>
-  <cellMetadata count="1">
-    <bk>
-      <rc t="1" v="0"/>
-    </bk>
-  </cellMetadata>
-</metadata>
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="8">
+  <si>
+    <t>Наименование</t>
+  </si>
+  <si>
+    <t>SKU</t>
+  </si>
+  <si>
+    <t>№</t>
+  </si>
+  <si>
+    <t>Штрихкод</t>
+  </si>
+  <si>
+    <t>Ед. изм.</t>
+  </si>
+  <si>
+    <t>Мин. ост.</t>
+  </si>
+  <si>
+    <t>Макс. ост.</t>
+  </si>
+  <si>
+    <t>Цена</t>
+  </si>
+</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
-  <numFmts count="1">
-    <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
-  </numFmts>
-  <fonts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -44,15 +59,21 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -60,18 +81,49 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Обычный" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -396,76 +448,884 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:H72"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="2.625" customWidth="1"/>
+    <col min="2" max="2" width="30.125" customWidth="1"/>
+    <col min="4" max="4" width="10.75" customWidth="1"/>
+    <col min="7" max="7" width="9.375" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>????????????</v>
-      </c>
-      <c r="B1" t="str">
-        <v>???????</v>
-      </c>
-      <c r="C1" t="str">
-        <v>????????</v>
-      </c>
-      <c r="D1" t="str">
-        <v>??.???.</v>
-      </c>
-      <c r="E1" t="str">
-        <v>??????? E (?????????????)</v>
-      </c>
-      <c r="F1" t="str">
-        <v>???.???????</v>
-      </c>
-      <c r="G1" t="str">
-        <v>??????? G (?????????????)</v>
-      </c>
-      <c r="H1" t="str">
-        <v>??????? H (?????????????)</v>
-      </c>
-      <c r="I1" t="str">
-        <v>????.???????</v>
-      </c>
-      <c r="J1" t="str">
-        <v>????</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>??????? 24V</v>
-      </c>
-      <c r="B2" t="str">
-        <v>ST-001</v>
-      </c>
-      <c r="C2" t="str">
-        <v>ST-001</v>
-      </c>
-      <c r="D2" t="str">
-        <v>??</v>
-      </c>
-      <c r="E2" t="str">
-        <v/>
-      </c>
-      <c r="F2">
+    <row r="1" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="G2" t="str">
-        <v/>
-      </c>
-      <c r="H2" t="str">
-        <v/>
-      </c>
-      <c r="I2">
+      <c r="B1" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="J2">
-        <v>2290</v>
-      </c>
-    </row>
+      <c r="G1" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A2" s="4">
+        <v>1</v>
+      </c>
+      <c r="B2" s="1"/>
+      <c r="C2" s="1"/>
+      <c r="D2" s="1"/>
+      <c r="E2" s="1"/>
+      <c r="F2" s="1"/>
+      <c r="G2" s="1"/>
+      <c r="H2" s="1"/>
+    </row>
+    <row r="3" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A3" s="4">
+        <v>2</v>
+      </c>
+      <c r="B3" s="1"/>
+      <c r="C3" s="1"/>
+      <c r="D3" s="1"/>
+      <c r="E3" s="1"/>
+      <c r="F3" s="1"/>
+      <c r="G3" s="1"/>
+      <c r="H3" s="1"/>
+    </row>
+    <row r="4" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A4" s="4">
+        <v>3</v>
+      </c>
+      <c r="B4" s="1"/>
+      <c r="C4" s="1"/>
+      <c r="D4" s="1"/>
+      <c r="E4" s="1"/>
+      <c r="F4" s="1"/>
+      <c r="G4" s="1"/>
+      <c r="H4" s="1"/>
+    </row>
+    <row r="5" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A5" s="4">
+        <v>4</v>
+      </c>
+      <c r="B5" s="1"/>
+      <c r="C5" s="1"/>
+      <c r="D5" s="1"/>
+      <c r="E5" s="1"/>
+      <c r="F5" s="1"/>
+      <c r="G5" s="1"/>
+      <c r="H5" s="1"/>
+    </row>
+    <row r="6" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A6" s="4">
+        <v>5</v>
+      </c>
+      <c r="B6" s="1"/>
+      <c r="C6" s="1"/>
+      <c r="D6" s="1"/>
+      <c r="E6" s="1"/>
+      <c r="F6" s="1"/>
+      <c r="G6" s="1"/>
+      <c r="H6" s="1"/>
+    </row>
+    <row r="7" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A7" s="4">
+        <v>6</v>
+      </c>
+      <c r="B7" s="1"/>
+      <c r="C7" s="1"/>
+      <c r="D7" s="1"/>
+      <c r="E7" s="1"/>
+      <c r="F7" s="1"/>
+      <c r="G7" s="1"/>
+      <c r="H7" s="1"/>
+    </row>
+    <row r="8" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A8" s="4">
+        <v>7</v>
+      </c>
+      <c r="B8" s="1"/>
+      <c r="C8" s="1"/>
+      <c r="D8" s="1"/>
+      <c r="E8" s="1"/>
+      <c r="F8" s="1"/>
+      <c r="G8" s="1"/>
+      <c r="H8" s="1"/>
+    </row>
+    <row r="9" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A9" s="4">
+        <v>8</v>
+      </c>
+      <c r="B9" s="1"/>
+      <c r="C9" s="1"/>
+      <c r="D9" s="1"/>
+      <c r="E9" s="1"/>
+      <c r="F9" s="1"/>
+      <c r="G9" s="1"/>
+      <c r="H9" s="1"/>
+    </row>
+    <row r="10" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A10" s="4">
+        <v>9</v>
+      </c>
+      <c r="B10" s="1"/>
+      <c r="C10" s="1"/>
+      <c r="D10" s="1"/>
+      <c r="E10" s="1"/>
+      <c r="F10" s="1"/>
+      <c r="G10" s="1"/>
+      <c r="H10" s="1"/>
+    </row>
+    <row r="11" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A11" s="4">
+        <v>10</v>
+      </c>
+      <c r="B11" s="1"/>
+      <c r="C11" s="1"/>
+      <c r="D11" s="1"/>
+      <c r="E11" s="1"/>
+      <c r="F11" s="1"/>
+      <c r="G11" s="1"/>
+      <c r="H11" s="1"/>
+    </row>
+    <row r="12" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A12" s="4">
+        <v>11</v>
+      </c>
+      <c r="B12" s="1"/>
+      <c r="C12" s="1"/>
+      <c r="D12" s="1"/>
+      <c r="E12" s="1"/>
+      <c r="F12" s="1"/>
+      <c r="G12" s="1"/>
+      <c r="H12" s="1"/>
+    </row>
+    <row r="13" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A13" s="4">
+        <v>12</v>
+      </c>
+      <c r="B13" s="1"/>
+      <c r="C13" s="1"/>
+      <c r="D13" s="1"/>
+      <c r="E13" s="1"/>
+      <c r="F13" s="1"/>
+      <c r="G13" s="1"/>
+      <c r="H13" s="1"/>
+    </row>
+    <row r="14" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A14" s="4">
+        <v>13</v>
+      </c>
+      <c r="B14" s="1"/>
+      <c r="C14" s="1"/>
+      <c r="D14" s="1"/>
+      <c r="E14" s="1"/>
+      <c r="F14" s="1"/>
+      <c r="G14" s="1"/>
+      <c r="H14" s="1"/>
+    </row>
+    <row r="15" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A15" s="4">
+        <v>14</v>
+      </c>
+      <c r="B15" s="1"/>
+      <c r="C15" s="1"/>
+      <c r="D15" s="1"/>
+      <c r="E15" s="1"/>
+      <c r="F15" s="1"/>
+      <c r="G15" s="1"/>
+      <c r="H15" s="1"/>
+    </row>
+    <row r="16" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A16" s="4">
+        <v>15</v>
+      </c>
+      <c r="B16" s="1"/>
+      <c r="C16" s="1"/>
+      <c r="D16" s="1"/>
+      <c r="E16" s="1"/>
+      <c r="F16" s="1"/>
+      <c r="G16" s="1"/>
+      <c r="H16" s="1"/>
+    </row>
+    <row r="17" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A17" s="4">
+        <v>16</v>
+      </c>
+      <c r="B17" s="1"/>
+      <c r="C17" s="1"/>
+      <c r="D17" s="1"/>
+      <c r="E17" s="1"/>
+      <c r="F17" s="1"/>
+      <c r="G17" s="1"/>
+      <c r="H17" s="1"/>
+    </row>
+    <row r="18" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A18" s="4">
+        <v>17</v>
+      </c>
+      <c r="B18" s="1"/>
+      <c r="C18" s="1"/>
+      <c r="D18" s="1"/>
+      <c r="E18" s="1"/>
+      <c r="F18" s="1"/>
+      <c r="G18" s="1"/>
+      <c r="H18" s="1"/>
+    </row>
+    <row r="19" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A19" s="4">
+        <v>18</v>
+      </c>
+      <c r="B19" s="1"/>
+      <c r="C19" s="1"/>
+      <c r="D19" s="1"/>
+      <c r="E19" s="1"/>
+      <c r="F19" s="1"/>
+      <c r="G19" s="1"/>
+      <c r="H19" s="1"/>
+    </row>
+    <row r="20" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A20" s="4">
+        <v>19</v>
+      </c>
+      <c r="B20" s="1"/>
+      <c r="C20" s="1"/>
+      <c r="D20" s="1"/>
+      <c r="E20" s="1"/>
+      <c r="F20" s="1"/>
+      <c r="G20" s="1"/>
+      <c r="H20" s="1"/>
+    </row>
+    <row r="21" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A21" s="4">
+        <v>20</v>
+      </c>
+      <c r="B21" s="1"/>
+      <c r="C21" s="1"/>
+      <c r="D21" s="1"/>
+      <c r="E21" s="1"/>
+      <c r="F21" s="1"/>
+      <c r="G21" s="1"/>
+      <c r="H21" s="1"/>
+    </row>
+    <row r="22" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A22" s="4">
+        <v>21</v>
+      </c>
+      <c r="B22" s="1"/>
+      <c r="C22" s="1"/>
+      <c r="D22" s="1"/>
+      <c r="E22" s="1"/>
+      <c r="F22" s="1"/>
+      <c r="G22" s="1"/>
+      <c r="H22" s="1"/>
+    </row>
+    <row r="23" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A23" s="4">
+        <v>22</v>
+      </c>
+      <c r="B23" s="1"/>
+      <c r="C23" s="1"/>
+      <c r="D23" s="1"/>
+      <c r="E23" s="1"/>
+      <c r="F23" s="1"/>
+      <c r="G23" s="1"/>
+      <c r="H23" s="1"/>
+    </row>
+    <row r="24" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A24" s="4">
+        <v>23</v>
+      </c>
+      <c r="B24" s="1"/>
+      <c r="C24" s="1"/>
+      <c r="D24" s="1"/>
+      <c r="E24" s="1"/>
+      <c r="F24" s="1"/>
+      <c r="G24" s="1"/>
+      <c r="H24" s="1"/>
+    </row>
+    <row r="25" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A25" s="4">
+        <v>24</v>
+      </c>
+      <c r="B25" s="1"/>
+      <c r="C25" s="1"/>
+      <c r="D25" s="1"/>
+      <c r="E25" s="1"/>
+      <c r="F25" s="1"/>
+      <c r="G25" s="1"/>
+      <c r="H25" s="1"/>
+    </row>
+    <row r="26" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A26" s="4">
+        <v>25</v>
+      </c>
+      <c r="B26" s="1"/>
+      <c r="C26" s="1"/>
+      <c r="D26" s="1"/>
+      <c r="E26" s="1"/>
+      <c r="F26" s="1"/>
+      <c r="G26" s="1"/>
+      <c r="H26" s="1"/>
+    </row>
+    <row r="27" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A27" s="4">
+        <v>26</v>
+      </c>
+      <c r="B27" s="1"/>
+      <c r="C27" s="1"/>
+      <c r="D27" s="1"/>
+      <c r="E27" s="1"/>
+      <c r="F27" s="1"/>
+      <c r="G27" s="1"/>
+      <c r="H27" s="1"/>
+    </row>
+    <row r="28" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A28" s="4">
+        <v>27</v>
+      </c>
+      <c r="B28" s="1"/>
+      <c r="C28" s="1"/>
+      <c r="D28" s="1"/>
+      <c r="E28" s="1"/>
+      <c r="F28" s="1"/>
+      <c r="G28" s="1"/>
+      <c r="H28" s="1"/>
+    </row>
+    <row r="29" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A29" s="4">
+        <v>28</v>
+      </c>
+      <c r="B29" s="1"/>
+      <c r="C29" s="1"/>
+      <c r="D29" s="1"/>
+      <c r="E29" s="1"/>
+      <c r="F29" s="1"/>
+      <c r="G29" s="1"/>
+      <c r="H29" s="1"/>
+    </row>
+    <row r="30" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A30" s="4">
+        <v>29</v>
+      </c>
+      <c r="B30" s="1"/>
+      <c r="C30" s="1"/>
+      <c r="D30" s="1"/>
+      <c r="E30" s="1"/>
+      <c r="F30" s="1"/>
+      <c r="G30" s="1"/>
+      <c r="H30" s="1"/>
+    </row>
+    <row r="31" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A31" s="4">
+        <v>30</v>
+      </c>
+      <c r="B31" s="1"/>
+      <c r="C31" s="1"/>
+      <c r="D31" s="1"/>
+      <c r="E31" s="1"/>
+      <c r="F31" s="1"/>
+      <c r="G31" s="1"/>
+      <c r="H31" s="1"/>
+    </row>
+    <row r="32" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A32" s="4">
+        <v>31</v>
+      </c>
+      <c r="B32" s="1"/>
+      <c r="C32" s="1"/>
+      <c r="D32" s="1"/>
+      <c r="E32" s="1"/>
+      <c r="F32" s="1"/>
+      <c r="G32" s="1"/>
+      <c r="H32" s="1"/>
+    </row>
+    <row r="33" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A33" s="4">
+        <v>32</v>
+      </c>
+      <c r="B33" s="1"/>
+      <c r="C33" s="1"/>
+      <c r="D33" s="1"/>
+      <c r="E33" s="1"/>
+      <c r="F33" s="1"/>
+      <c r="G33" s="1"/>
+      <c r="H33" s="1"/>
+    </row>
+    <row r="34" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A34" s="4">
+        <v>33</v>
+      </c>
+      <c r="B34" s="1"/>
+      <c r="C34" s="1"/>
+      <c r="D34" s="1"/>
+      <c r="E34" s="1"/>
+      <c r="F34" s="1"/>
+      <c r="G34" s="1"/>
+      <c r="H34" s="1"/>
+    </row>
+    <row r="35" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A35" s="4">
+        <v>34</v>
+      </c>
+      <c r="B35" s="1"/>
+      <c r="C35" s="1"/>
+      <c r="D35" s="1"/>
+      <c r="E35" s="1"/>
+      <c r="F35" s="1"/>
+      <c r="G35" s="1"/>
+      <c r="H35" s="1"/>
+    </row>
+    <row r="36" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A36" s="4">
+        <v>35</v>
+      </c>
+      <c r="B36" s="1"/>
+      <c r="C36" s="1"/>
+      <c r="D36" s="1"/>
+      <c r="E36" s="1"/>
+      <c r="F36" s="1"/>
+      <c r="G36" s="1"/>
+      <c r="H36" s="1"/>
+    </row>
+    <row r="37" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A37" s="4">
+        <v>36</v>
+      </c>
+      <c r="B37" s="1"/>
+      <c r="C37" s="1"/>
+      <c r="D37" s="1"/>
+      <c r="E37" s="1"/>
+      <c r="F37" s="1"/>
+      <c r="G37" s="1"/>
+      <c r="H37" s="1"/>
+    </row>
+    <row r="38" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A38" s="4">
+        <v>37</v>
+      </c>
+      <c r="B38" s="1"/>
+      <c r="C38" s="1"/>
+      <c r="D38" s="1"/>
+      <c r="E38" s="1"/>
+      <c r="F38" s="1"/>
+      <c r="G38" s="1"/>
+      <c r="H38" s="1"/>
+    </row>
+    <row r="39" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A39" s="4">
+        <v>38</v>
+      </c>
+      <c r="B39" s="1"/>
+      <c r="C39" s="1"/>
+      <c r="D39" s="1"/>
+      <c r="E39" s="1"/>
+      <c r="F39" s="1"/>
+      <c r="G39" s="1"/>
+      <c r="H39" s="1"/>
+    </row>
+    <row r="40" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A40" s="4">
+        <v>39</v>
+      </c>
+      <c r="B40" s="1"/>
+      <c r="C40" s="1"/>
+      <c r="D40" s="1"/>
+      <c r="E40" s="1"/>
+      <c r="F40" s="1"/>
+      <c r="G40" s="1"/>
+      <c r="H40" s="1"/>
+    </row>
+    <row r="41" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A41" s="4">
+        <v>40</v>
+      </c>
+      <c r="B41" s="1"/>
+      <c r="C41" s="1"/>
+      <c r="D41" s="1"/>
+      <c r="E41" s="1"/>
+      <c r="F41" s="1"/>
+      <c r="G41" s="1"/>
+      <c r="H41" s="1"/>
+    </row>
+    <row r="42" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A42" s="4">
+        <v>41</v>
+      </c>
+      <c r="B42" s="1"/>
+      <c r="C42" s="1"/>
+      <c r="D42" s="1"/>
+      <c r="E42" s="1"/>
+      <c r="F42" s="1"/>
+      <c r="G42" s="1"/>
+      <c r="H42" s="1"/>
+    </row>
+    <row r="43" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A43" s="4">
+        <v>42</v>
+      </c>
+      <c r="B43" s="1"/>
+      <c r="C43" s="1"/>
+      <c r="D43" s="1"/>
+      <c r="E43" s="1"/>
+      <c r="F43" s="1"/>
+      <c r="G43" s="1"/>
+      <c r="H43" s="1"/>
+    </row>
+    <row r="44" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A44" s="4">
+        <v>43</v>
+      </c>
+      <c r="B44" s="1"/>
+      <c r="C44" s="1"/>
+      <c r="D44" s="1"/>
+      <c r="E44" s="1"/>
+      <c r="F44" s="1"/>
+      <c r="G44" s="1"/>
+      <c r="H44" s="1"/>
+    </row>
+    <row r="45" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A45" s="4">
+        <v>44</v>
+      </c>
+      <c r="B45" s="1"/>
+      <c r="C45" s="1"/>
+      <c r="D45" s="1"/>
+      <c r="E45" s="1"/>
+      <c r="F45" s="1"/>
+      <c r="G45" s="1"/>
+      <c r="H45" s="1"/>
+    </row>
+    <row r="46" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A46" s="4">
+        <v>45</v>
+      </c>
+      <c r="B46" s="1"/>
+      <c r="C46" s="1"/>
+      <c r="D46" s="1"/>
+      <c r="E46" s="1"/>
+      <c r="F46" s="1"/>
+      <c r="G46" s="1"/>
+      <c r="H46" s="1"/>
+    </row>
+    <row r="47" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A47" s="4">
+        <v>46</v>
+      </c>
+      <c r="B47" s="1"/>
+      <c r="C47" s="1"/>
+      <c r="D47" s="1"/>
+      <c r="E47" s="1"/>
+      <c r="F47" s="1"/>
+      <c r="G47" s="1"/>
+      <c r="H47" s="1"/>
+    </row>
+    <row r="48" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A48" s="4">
+        <v>47</v>
+      </c>
+      <c r="B48" s="1"/>
+      <c r="C48" s="1"/>
+      <c r="D48" s="1"/>
+      <c r="E48" s="1"/>
+      <c r="F48" s="1"/>
+      <c r="G48" s="1"/>
+      <c r="H48" s="1"/>
+    </row>
+    <row r="49" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A49" s="4">
+        <v>48</v>
+      </c>
+      <c r="B49" s="1"/>
+      <c r="C49" s="1"/>
+      <c r="D49" s="1"/>
+      <c r="E49" s="1"/>
+      <c r="F49" s="1"/>
+      <c r="G49" s="1"/>
+      <c r="H49" s="1"/>
+    </row>
+    <row r="50" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A50" s="4">
+        <v>49</v>
+      </c>
+      <c r="B50" s="1"/>
+      <c r="C50" s="1"/>
+      <c r="D50" s="1"/>
+      <c r="E50" s="1"/>
+      <c r="F50" s="1"/>
+      <c r="G50" s="1"/>
+      <c r="H50" s="1"/>
+    </row>
+    <row r="51" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A51" s="4">
+        <v>50</v>
+      </c>
+      <c r="B51" s="1"/>
+      <c r="C51" s="1"/>
+      <c r="D51" s="1"/>
+      <c r="E51" s="1"/>
+      <c r="F51" s="1"/>
+      <c r="G51" s="1"/>
+      <c r="H51" s="1"/>
+    </row>
+    <row r="52" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A52" s="4">
+        <v>51</v>
+      </c>
+      <c r="B52" s="1"/>
+      <c r="C52" s="1"/>
+      <c r="D52" s="1"/>
+      <c r="E52" s="1"/>
+      <c r="F52" s="1"/>
+      <c r="G52" s="1"/>
+      <c r="H52" s="1"/>
+    </row>
+    <row r="53" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A53" s="4">
+        <v>52</v>
+      </c>
+      <c r="B53" s="1"/>
+      <c r="C53" s="1"/>
+      <c r="D53" s="1"/>
+      <c r="E53" s="1"/>
+      <c r="F53" s="1"/>
+      <c r="G53" s="1"/>
+      <c r="H53" s="1"/>
+    </row>
+    <row r="54" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A54" s="4">
+        <v>53</v>
+      </c>
+      <c r="B54" s="1"/>
+      <c r="C54" s="1"/>
+      <c r="D54" s="1"/>
+      <c r="E54" s="1"/>
+      <c r="F54" s="1"/>
+      <c r="G54" s="1"/>
+      <c r="H54" s="1"/>
+    </row>
+    <row r="55" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A55" s="4">
+        <v>54</v>
+      </c>
+      <c r="B55" s="1"/>
+      <c r="C55" s="1"/>
+      <c r="D55" s="1"/>
+      <c r="E55" s="1"/>
+      <c r="F55" s="1"/>
+      <c r="G55" s="1"/>
+      <c r="H55" s="1"/>
+    </row>
+    <row r="56" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A56" s="4">
+        <v>55</v>
+      </c>
+      <c r="B56" s="1"/>
+      <c r="C56" s="1"/>
+      <c r="D56" s="1"/>
+      <c r="E56" s="1"/>
+      <c r="F56" s="1"/>
+      <c r="G56" s="1"/>
+      <c r="H56" s="1"/>
+    </row>
+    <row r="57" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A57" s="4">
+        <v>56</v>
+      </c>
+      <c r="B57" s="1"/>
+      <c r="C57" s="1"/>
+      <c r="D57" s="1"/>
+      <c r="E57" s="1"/>
+      <c r="F57" s="1"/>
+      <c r="G57" s="1"/>
+      <c r="H57" s="1"/>
+    </row>
+    <row r="58" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A58" s="4">
+        <v>57</v>
+      </c>
+      <c r="B58" s="1"/>
+      <c r="C58" s="1"/>
+      <c r="D58" s="1"/>
+      <c r="E58" s="1"/>
+      <c r="F58" s="1"/>
+      <c r="G58" s="1"/>
+      <c r="H58" s="1"/>
+    </row>
+    <row r="59" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A59" s="4">
+        <v>58</v>
+      </c>
+      <c r="B59" s="1"/>
+      <c r="C59" s="1"/>
+      <c r="D59" s="1"/>
+      <c r="E59" s="1"/>
+      <c r="F59" s="1"/>
+      <c r="G59" s="1"/>
+      <c r="H59" s="1"/>
+    </row>
+    <row r="60" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A60" s="4">
+        <v>59</v>
+      </c>
+      <c r="B60" s="1"/>
+      <c r="C60" s="1"/>
+      <c r="D60" s="1"/>
+      <c r="E60" s="1"/>
+      <c r="F60" s="1"/>
+      <c r="G60" s="1"/>
+      <c r="H60" s="1"/>
+    </row>
+    <row r="61" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A61" s="4">
+        <v>60</v>
+      </c>
+      <c r="B61" s="1"/>
+      <c r="C61" s="1"/>
+      <c r="D61" s="1"/>
+      <c r="E61" s="1"/>
+      <c r="F61" s="1"/>
+      <c r="G61" s="1"/>
+      <c r="H61" s="1"/>
+    </row>
+    <row r="62" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A62" s="4">
+        <v>61</v>
+      </c>
+      <c r="B62" s="1"/>
+      <c r="C62" s="1"/>
+      <c r="D62" s="1"/>
+      <c r="E62" s="1"/>
+      <c r="F62" s="1"/>
+      <c r="G62" s="1"/>
+      <c r="H62" s="1"/>
+    </row>
+    <row r="63" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A63" s="4">
+        <v>62</v>
+      </c>
+      <c r="B63" s="1"/>
+      <c r="C63" s="1"/>
+      <c r="D63" s="1"/>
+      <c r="E63" s="1"/>
+      <c r="F63" s="1"/>
+      <c r="G63" s="1"/>
+      <c r="H63" s="1"/>
+    </row>
+    <row r="64" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A64" s="4">
+        <v>63</v>
+      </c>
+      <c r="B64" s="1"/>
+      <c r="C64" s="1"/>
+      <c r="D64" s="1"/>
+      <c r="E64" s="1"/>
+      <c r="F64" s="1"/>
+      <c r="G64" s="1"/>
+      <c r="H64" s="1"/>
+    </row>
+    <row r="65" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A65" s="4">
+        <v>64</v>
+      </c>
+      <c r="B65" s="1"/>
+      <c r="C65" s="1"/>
+      <c r="D65" s="1"/>
+      <c r="E65" s="1"/>
+      <c r="F65" s="1"/>
+      <c r="G65" s="1"/>
+      <c r="H65" s="1"/>
+    </row>
+    <row r="66" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A66" s="4">
+        <v>65</v>
+      </c>
+      <c r="B66" s="1"/>
+      <c r="C66" s="1"/>
+      <c r="D66" s="1"/>
+      <c r="E66" s="1"/>
+      <c r="F66" s="1"/>
+      <c r="G66" s="1"/>
+      <c r="H66" s="1"/>
+    </row>
+    <row r="67" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A67" s="4">
+        <v>66</v>
+      </c>
+      <c r="B67" s="1"/>
+      <c r="C67" s="1"/>
+      <c r="D67" s="1"/>
+      <c r="E67" s="1"/>
+      <c r="F67" s="1"/>
+      <c r="G67" s="1"/>
+      <c r="H67" s="1"/>
+    </row>
+    <row r="68" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A68" s="4">
+        <v>67</v>
+      </c>
+      <c r="B68" s="1"/>
+      <c r="C68" s="1"/>
+      <c r="D68" s="1"/>
+      <c r="E68" s="1"/>
+      <c r="F68" s="1"/>
+      <c r="G68" s="1"/>
+      <c r="H68" s="1"/>
+    </row>
+    <row r="69" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A69" s="4">
+        <v>68</v>
+      </c>
+      <c r="B69" s="1"/>
+      <c r="C69" s="1"/>
+      <c r="D69" s="1"/>
+      <c r="E69" s="1"/>
+      <c r="F69" s="1"/>
+      <c r="G69" s="1"/>
+      <c r="H69" s="1"/>
+    </row>
+    <row r="70" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A70" s="4">
+        <v>69</v>
+      </c>
+      <c r="B70" s="1"/>
+      <c r="C70" s="1"/>
+      <c r="D70" s="1"/>
+      <c r="E70" s="1"/>
+      <c r="F70" s="1"/>
+      <c r="G70" s="1"/>
+      <c r="H70" s="1"/>
+    </row>
+    <row r="71" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A71" s="4">
+        <v>70</v>
+      </c>
+      <c r="B71" s="1"/>
+      <c r="C71" s="1"/>
+      <c r="D71" s="1"/>
+      <c r="E71" s="1"/>
+      <c r="F71" s="1"/>
+      <c r="G71" s="1"/>
+      <c r="H71" s="1"/>
+    </row>
+    <row r="72" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
   </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:J2"/>
-  </ignoredErrors>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>